<commit_message>
Group packing fields; simpler registration; flexible web addresses
</commit_message>
<xml_diff>
--- a/public/Lulyboo_Supplier_Product_Template.xlsx
+++ b/public/Lulyboo_Supplier_Product_Template.xlsx
@@ -480,7 +480,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AJ203"/>
+  <dimension ref="A1:AI203"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -506,19 +506,18 @@
     <col width="25" customWidth="1" min="21" max="21"/>
     <col width="29" customWidth="1" min="22" max="22"/>
     <col width="19" customWidth="1" min="23" max="23"/>
-    <col width="24" customWidth="1" min="24" max="24"/>
-    <col width="22" customWidth="1" min="25" max="25"/>
-    <col width="25" customWidth="1" min="26" max="26"/>
-    <col width="20" customWidth="1" min="27" max="27"/>
-    <col width="19" customWidth="1" min="28" max="28"/>
-    <col width="20" customWidth="1" min="29" max="29"/>
-    <col width="24" customWidth="1" min="30" max="30"/>
-    <col width="26" customWidth="1" min="31" max="31"/>
+    <col width="22" customWidth="1" min="24" max="24"/>
+    <col width="25" customWidth="1" min="25" max="25"/>
+    <col width="20" customWidth="1" min="26" max="26"/>
+    <col width="19" customWidth="1" min="27" max="27"/>
+    <col width="20" customWidth="1" min="28" max="28"/>
+    <col width="24" customWidth="1" min="29" max="29"/>
+    <col width="26" customWidth="1" min="30" max="30"/>
+    <col width="22" customWidth="1" min="31" max="31"/>
     <col width="22" customWidth="1" min="32" max="32"/>
     <col width="22" customWidth="1" min="33" max="33"/>
-    <col width="22" customWidth="1" min="34" max="34"/>
-    <col width="12" customWidth="1" min="35" max="35"/>
-    <col width="15" customWidth="1" min="36" max="36"/>
+    <col width="12" customWidth="1" min="34" max="34"/>
+    <col width="15" customWidth="1" min="35" max="35"/>
   </cols>
   <sheetData>
     <row r="1" ht="34" customHeight="1">
@@ -639,65 +638,60 @@
       </c>
       <c r="X1" s="1" t="inlineStr">
         <is>
-          <t>Suggested Retail (USD)</t>
+          <t>Units per Inner Pack</t>
         </is>
       </c>
       <c r="Y1" s="1" t="inlineStr">
         <is>
-          <t>Units per Inner Pack</t>
+          <t>Units per Master Carton</t>
         </is>
       </c>
       <c r="Z1" s="1" t="inlineStr">
         <is>
-          <t>Units per Master Carton</t>
+          <t>Carton Length (cm)</t>
         </is>
       </c>
       <c r="AA1" s="1" t="inlineStr">
         <is>
-          <t>Carton Length (cm)</t>
+          <t>Carton Width (cm)</t>
         </is>
       </c>
       <c r="AB1" s="1" t="inlineStr">
         <is>
-          <t>Carton Width (cm)</t>
+          <t>Carton Height (cm)</t>
         </is>
       </c>
       <c r="AC1" s="1" t="inlineStr">
         <is>
-          <t>Carton Height (cm)</t>
+          <t>Carton Net Weight (kg)</t>
         </is>
       </c>
       <c r="AD1" s="1" t="inlineStr">
         <is>
-          <t>Carton Net Weight (kg)</t>
+          <t>Carton Gross Weight (kg)</t>
         </is>
       </c>
       <c r="AE1" s="1" t="inlineStr">
         <is>
-          <t>Carton Gross Weight (kg)</t>
+          <t>Qty per 20GP (units)</t>
         </is>
       </c>
       <c r="AF1" s="1" t="inlineStr">
         <is>
-          <t>Qty per 20GP (units)</t>
+          <t>Qty per 40GP (units)</t>
         </is>
       </c>
       <c r="AG1" s="1" t="inlineStr">
         <is>
-          <t>Qty per 40GP (units)</t>
+          <t>Qty per 40HQ (units)</t>
         </is>
       </c>
       <c r="AH1" s="1" t="inlineStr">
         <is>
-          <t>Qty per 40HQ (units)</t>
+          <t>Photo Link</t>
         </is>
       </c>
       <c r="AI1" s="1" t="inlineStr">
-        <is>
-          <t>Photo Link</t>
-        </is>
-      </c>
-      <c r="AJ1" s="1" t="inlineStr">
         <is>
           <t>Factory Notes</t>
         </is>
@@ -821,65 +815,60 @@
       </c>
       <c r="X2" s="2" t="inlineStr">
         <is>
-          <t>建议零售价（USD）</t>
+          <t>内盒装数（件）</t>
         </is>
       </c>
       <c r="Y2" s="2" t="inlineStr">
         <is>
-          <t>内盒装数（件）</t>
+          <t>外箱装数（件/箱）</t>
         </is>
       </c>
       <c r="Z2" s="2" t="inlineStr">
         <is>
-          <t>外箱装数（件/箱）</t>
+          <t>外箱长（cm）</t>
         </is>
       </c>
       <c r="AA2" s="2" t="inlineStr">
         <is>
-          <t>外箱长（cm）</t>
+          <t>外箱宽（cm）</t>
         </is>
       </c>
       <c r="AB2" s="2" t="inlineStr">
         <is>
-          <t>外箱宽（cm）</t>
+          <t>外箱高（cm）</t>
         </is>
       </c>
       <c r="AC2" s="2" t="inlineStr">
         <is>
-          <t>外箱高（cm）</t>
+          <t>外箱净重（kg）</t>
         </is>
       </c>
       <c r="AD2" s="2" t="inlineStr">
         <is>
-          <t>外箱净重（kg）</t>
+          <t>外箱毛重（kg）</t>
         </is>
       </c>
       <c r="AE2" s="2" t="inlineStr">
         <is>
-          <t>外箱毛重（kg）</t>
+          <t>20GP 装柜数量（件，选填）</t>
         </is>
       </c>
       <c r="AF2" s="2" t="inlineStr">
         <is>
-          <t>20GP 装柜数量（件，选填）</t>
+          <t>40GP 装柜数量（件，选填）</t>
         </is>
       </c>
       <c r="AG2" s="2" t="inlineStr">
         <is>
-          <t>40GP 装柜数量（件，选填）</t>
+          <t>40HQ 装柜数量（件，选填）</t>
         </is>
       </c>
       <c r="AH2" s="2" t="inlineStr">
         <is>
-          <t>40HQ 装柜数量（件，选填）</t>
+          <t>图片 / 目录链接</t>
         </is>
       </c>
       <c r="AI2" s="2" t="inlineStr">
-        <is>
-          <t>图片 / 目录链接</t>
-        </is>
-      </c>
-      <c r="AJ2" s="2" t="inlineStr">
         <is>
           <t>工厂备注</t>
         </is>
@@ -992,44 +981,41 @@
         </is>
       </c>
       <c r="X3" s="3" t="n">
-        <v>14.99</v>
+        <v>6</v>
       </c>
       <c r="Y3" s="3" t="n">
-        <v>6</v>
+        <v>24</v>
       </c>
       <c r="Z3" s="3" t="n">
-        <v>24</v>
+        <v>50</v>
       </c>
       <c r="AA3" s="3" t="n">
-        <v>50</v>
+        <v>35</v>
       </c>
       <c r="AB3" s="3" t="n">
-        <v>35</v>
+        <v>30</v>
       </c>
       <c r="AC3" s="3" t="n">
-        <v>30</v>
+        <v>9.6</v>
       </c>
       <c r="AD3" s="3" t="n">
-        <v>9.6</v>
+        <v>10.6</v>
       </c>
       <c r="AE3" s="3" t="n">
-        <v>10.6</v>
+        <v>11088</v>
       </c>
       <c r="AF3" s="3" t="n">
-        <v>11088</v>
+        <v>24192</v>
       </c>
       <c r="AG3" s="3" t="n">
-        <v>24192</v>
-      </c>
-      <c r="AH3" s="3" t="n">
         <v>28800</v>
       </c>
-      <c r="AI3" s="3" t="inlineStr">
+      <c r="AH3" s="3" t="inlineStr">
         <is>
           <t>https://example.com/photo.jpg</t>
         </is>
       </c>
-      <c r="AJ3" s="3" t="inlineStr"/>
+      <c r="AI3" s="3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="5" t="n"/>
@@ -1067,7 +1053,6 @@
       <c r="AG4" s="5" t="n"/>
       <c r="AH4" s="5" t="n"/>
       <c r="AI4" s="5" t="n"/>
-      <c r="AJ4" s="5" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="5" t="n"/>
@@ -1105,7 +1090,6 @@
       <c r="AG5" s="5" t="n"/>
       <c r="AH5" s="5" t="n"/>
       <c r="AI5" s="5" t="n"/>
-      <c r="AJ5" s="5" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="5" t="n"/>
@@ -1143,7 +1127,6 @@
       <c r="AG6" s="5" t="n"/>
       <c r="AH6" s="5" t="n"/>
       <c r="AI6" s="5" t="n"/>
-      <c r="AJ6" s="5" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="5" t="n"/>
@@ -1181,7 +1164,6 @@
       <c r="AG7" s="5" t="n"/>
       <c r="AH7" s="5" t="n"/>
       <c r="AI7" s="5" t="n"/>
-      <c r="AJ7" s="5" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="5" t="n"/>
@@ -1219,7 +1201,6 @@
       <c r="AG8" s="5" t="n"/>
       <c r="AH8" s="5" t="n"/>
       <c r="AI8" s="5" t="n"/>
-      <c r="AJ8" s="5" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="5" t="n"/>
@@ -1257,7 +1238,6 @@
       <c r="AG9" s="5" t="n"/>
       <c r="AH9" s="5" t="n"/>
       <c r="AI9" s="5" t="n"/>
-      <c r="AJ9" s="5" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="5" t="n"/>
@@ -1295,7 +1275,6 @@
       <c r="AG10" s="5" t="n"/>
       <c r="AH10" s="5" t="n"/>
       <c r="AI10" s="5" t="n"/>
-      <c r="AJ10" s="5" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="5" t="n"/>
@@ -1333,7 +1312,6 @@
       <c r="AG11" s="5" t="n"/>
       <c r="AH11" s="5" t="n"/>
       <c r="AI11" s="5" t="n"/>
-      <c r="AJ11" s="5" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="5" t="n"/>
@@ -1371,7 +1349,6 @@
       <c r="AG12" s="5" t="n"/>
       <c r="AH12" s="5" t="n"/>
       <c r="AI12" s="5" t="n"/>
-      <c r="AJ12" s="5" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="5" t="n"/>
@@ -1409,7 +1386,6 @@
       <c r="AG13" s="5" t="n"/>
       <c r="AH13" s="5" t="n"/>
       <c r="AI13" s="5" t="n"/>
-      <c r="AJ13" s="5" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="5" t="n"/>
@@ -1447,7 +1423,6 @@
       <c r="AG14" s="5" t="n"/>
       <c r="AH14" s="5" t="n"/>
       <c r="AI14" s="5" t="n"/>
-      <c r="AJ14" s="5" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="5" t="n"/>
@@ -1485,7 +1460,6 @@
       <c r="AG15" s="5" t="n"/>
       <c r="AH15" s="5" t="n"/>
       <c r="AI15" s="5" t="n"/>
-      <c r="AJ15" s="5" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="5" t="n"/>
@@ -1523,7 +1497,6 @@
       <c r="AG16" s="5" t="n"/>
       <c r="AH16" s="5" t="n"/>
       <c r="AI16" s="5" t="n"/>
-      <c r="AJ16" s="5" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="5" t="n"/>
@@ -1561,7 +1534,6 @@
       <c r="AG17" s="5" t="n"/>
       <c r="AH17" s="5" t="n"/>
       <c r="AI17" s="5" t="n"/>
-      <c r="AJ17" s="5" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="5" t="n"/>
@@ -1599,7 +1571,6 @@
       <c r="AG18" s="5" t="n"/>
       <c r="AH18" s="5" t="n"/>
       <c r="AI18" s="5" t="n"/>
-      <c r="AJ18" s="5" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="5" t="n"/>
@@ -1637,7 +1608,6 @@
       <c r="AG19" s="5" t="n"/>
       <c r="AH19" s="5" t="n"/>
       <c r="AI19" s="5" t="n"/>
-      <c r="AJ19" s="5" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="5" t="n"/>
@@ -1675,7 +1645,6 @@
       <c r="AG20" s="5" t="n"/>
       <c r="AH20" s="5" t="n"/>
       <c r="AI20" s="5" t="n"/>
-      <c r="AJ20" s="5" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="5" t="n"/>
@@ -1713,7 +1682,6 @@
       <c r="AG21" s="5" t="n"/>
       <c r="AH21" s="5" t="n"/>
       <c r="AI21" s="5" t="n"/>
-      <c r="AJ21" s="5" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="5" t="n"/>
@@ -1751,7 +1719,6 @@
       <c r="AG22" s="5" t="n"/>
       <c r="AH22" s="5" t="n"/>
       <c r="AI22" s="5" t="n"/>
-      <c r="AJ22" s="5" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="5" t="n"/>
@@ -1789,7 +1756,6 @@
       <c r="AG23" s="5" t="n"/>
       <c r="AH23" s="5" t="n"/>
       <c r="AI23" s="5" t="n"/>
-      <c r="AJ23" s="5" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="5" t="n"/>
@@ -1827,7 +1793,6 @@
       <c r="AG24" s="5" t="n"/>
       <c r="AH24" s="5" t="n"/>
       <c r="AI24" s="5" t="n"/>
-      <c r="AJ24" s="5" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="5" t="n"/>
@@ -1865,7 +1830,6 @@
       <c r="AG25" s="5" t="n"/>
       <c r="AH25" s="5" t="n"/>
       <c r="AI25" s="5" t="n"/>
-      <c r="AJ25" s="5" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="5" t="n"/>
@@ -1903,7 +1867,6 @@
       <c r="AG26" s="5" t="n"/>
       <c r="AH26" s="5" t="n"/>
       <c r="AI26" s="5" t="n"/>
-      <c r="AJ26" s="5" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="5" t="n"/>
@@ -1941,7 +1904,6 @@
       <c r="AG27" s="5" t="n"/>
       <c r="AH27" s="5" t="n"/>
       <c r="AI27" s="5" t="n"/>
-      <c r="AJ27" s="5" t="n"/>
     </row>
     <row r="28">
       <c r="A28" s="5" t="n"/>
@@ -1979,7 +1941,6 @@
       <c r="AG28" s="5" t="n"/>
       <c r="AH28" s="5" t="n"/>
       <c r="AI28" s="5" t="n"/>
-      <c r="AJ28" s="5" t="n"/>
     </row>
     <row r="29">
       <c r="A29" s="5" t="n"/>
@@ -2017,7 +1978,6 @@
       <c r="AG29" s="5" t="n"/>
       <c r="AH29" s="5" t="n"/>
       <c r="AI29" s="5" t="n"/>
-      <c r="AJ29" s="5" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="5" t="n"/>
@@ -2055,7 +2015,6 @@
       <c r="AG30" s="5" t="n"/>
       <c r="AH30" s="5" t="n"/>
       <c r="AI30" s="5" t="n"/>
-      <c r="AJ30" s="5" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="5" t="n"/>
@@ -2093,7 +2052,6 @@
       <c r="AG31" s="5" t="n"/>
       <c r="AH31" s="5" t="n"/>
       <c r="AI31" s="5" t="n"/>
-      <c r="AJ31" s="5" t="n"/>
     </row>
     <row r="32">
       <c r="A32" s="5" t="n"/>
@@ -2131,7 +2089,6 @@
       <c r="AG32" s="5" t="n"/>
       <c r="AH32" s="5" t="n"/>
       <c r="AI32" s="5" t="n"/>
-      <c r="AJ32" s="5" t="n"/>
     </row>
     <row r="33">
       <c r="A33" s="5" t="n"/>
@@ -2169,7 +2126,6 @@
       <c r="AG33" s="5" t="n"/>
       <c r="AH33" s="5" t="n"/>
       <c r="AI33" s="5" t="n"/>
-      <c r="AJ33" s="5" t="n"/>
     </row>
     <row r="34">
       <c r="A34" s="5" t="n"/>
@@ -2207,7 +2163,6 @@
       <c r="AG34" s="5" t="n"/>
       <c r="AH34" s="5" t="n"/>
       <c r="AI34" s="5" t="n"/>
-      <c r="AJ34" s="5" t="n"/>
     </row>
     <row r="35">
       <c r="A35" s="5" t="n"/>
@@ -2245,7 +2200,6 @@
       <c r="AG35" s="5" t="n"/>
       <c r="AH35" s="5" t="n"/>
       <c r="AI35" s="5" t="n"/>
-      <c r="AJ35" s="5" t="n"/>
     </row>
     <row r="36">
       <c r="A36" s="5" t="n"/>
@@ -2283,7 +2237,6 @@
       <c r="AG36" s="5" t="n"/>
       <c r="AH36" s="5" t="n"/>
       <c r="AI36" s="5" t="n"/>
-      <c r="AJ36" s="5" t="n"/>
     </row>
     <row r="37">
       <c r="A37" s="5" t="n"/>
@@ -2321,7 +2274,6 @@
       <c r="AG37" s="5" t="n"/>
       <c r="AH37" s="5" t="n"/>
       <c r="AI37" s="5" t="n"/>
-      <c r="AJ37" s="5" t="n"/>
     </row>
     <row r="38">
       <c r="A38" s="5" t="n"/>
@@ -2359,7 +2311,6 @@
       <c r="AG38" s="5" t="n"/>
       <c r="AH38" s="5" t="n"/>
       <c r="AI38" s="5" t="n"/>
-      <c r="AJ38" s="5" t="n"/>
     </row>
     <row r="39">
       <c r="A39" s="5" t="n"/>
@@ -2397,7 +2348,6 @@
       <c r="AG39" s="5" t="n"/>
       <c r="AH39" s="5" t="n"/>
       <c r="AI39" s="5" t="n"/>
-      <c r="AJ39" s="5" t="n"/>
     </row>
     <row r="40">
       <c r="A40" s="5" t="n"/>
@@ -2435,7 +2385,6 @@
       <c r="AG40" s="5" t="n"/>
       <c r="AH40" s="5" t="n"/>
       <c r="AI40" s="5" t="n"/>
-      <c r="AJ40" s="5" t="n"/>
     </row>
     <row r="41">
       <c r="A41" s="5" t="n"/>
@@ -2473,7 +2422,6 @@
       <c r="AG41" s="5" t="n"/>
       <c r="AH41" s="5" t="n"/>
       <c r="AI41" s="5" t="n"/>
-      <c r="AJ41" s="5" t="n"/>
     </row>
     <row r="42">
       <c r="A42" s="5" t="n"/>
@@ -2511,7 +2459,6 @@
       <c r="AG42" s="5" t="n"/>
       <c r="AH42" s="5" t="n"/>
       <c r="AI42" s="5" t="n"/>
-      <c r="AJ42" s="5" t="n"/>
     </row>
     <row r="43">
       <c r="A43" s="5" t="n"/>
@@ -2549,7 +2496,6 @@
       <c r="AG43" s="5" t="n"/>
       <c r="AH43" s="5" t="n"/>
       <c r="AI43" s="5" t="n"/>
-      <c r="AJ43" s="5" t="n"/>
     </row>
     <row r="44">
       <c r="A44" s="5" t="n"/>
@@ -2587,7 +2533,6 @@
       <c r="AG44" s="5" t="n"/>
       <c r="AH44" s="5" t="n"/>
       <c r="AI44" s="5" t="n"/>
-      <c r="AJ44" s="5" t="n"/>
     </row>
     <row r="45">
       <c r="A45" s="5" t="n"/>
@@ -2625,7 +2570,6 @@
       <c r="AG45" s="5" t="n"/>
       <c r="AH45" s="5" t="n"/>
       <c r="AI45" s="5" t="n"/>
-      <c r="AJ45" s="5" t="n"/>
     </row>
     <row r="46">
       <c r="A46" s="5" t="n"/>
@@ -2663,7 +2607,6 @@
       <c r="AG46" s="5" t="n"/>
       <c r="AH46" s="5" t="n"/>
       <c r="AI46" s="5" t="n"/>
-      <c r="AJ46" s="5" t="n"/>
     </row>
     <row r="47">
       <c r="A47" s="5" t="n"/>
@@ -2701,7 +2644,6 @@
       <c r="AG47" s="5" t="n"/>
       <c r="AH47" s="5" t="n"/>
       <c r="AI47" s="5" t="n"/>
-      <c r="AJ47" s="5" t="n"/>
     </row>
     <row r="48">
       <c r="A48" s="5" t="n"/>
@@ -2739,7 +2681,6 @@
       <c r="AG48" s="5" t="n"/>
       <c r="AH48" s="5" t="n"/>
       <c r="AI48" s="5" t="n"/>
-      <c r="AJ48" s="5" t="n"/>
     </row>
     <row r="49">
       <c r="A49" s="5" t="n"/>
@@ -2777,7 +2718,6 @@
       <c r="AG49" s="5" t="n"/>
       <c r="AH49" s="5" t="n"/>
       <c r="AI49" s="5" t="n"/>
-      <c r="AJ49" s="5" t="n"/>
     </row>
     <row r="50">
       <c r="A50" s="5" t="n"/>
@@ -2815,7 +2755,6 @@
       <c r="AG50" s="5" t="n"/>
       <c r="AH50" s="5" t="n"/>
       <c r="AI50" s="5" t="n"/>
-      <c r="AJ50" s="5" t="n"/>
     </row>
     <row r="51">
       <c r="A51" s="5" t="n"/>
@@ -2853,7 +2792,6 @@
       <c r="AG51" s="5" t="n"/>
       <c r="AH51" s="5" t="n"/>
       <c r="AI51" s="5" t="n"/>
-      <c r="AJ51" s="5" t="n"/>
     </row>
     <row r="52">
       <c r="A52" s="5" t="n"/>
@@ -2891,7 +2829,6 @@
       <c r="AG52" s="5" t="n"/>
       <c r="AH52" s="5" t="n"/>
       <c r="AI52" s="5" t="n"/>
-      <c r="AJ52" s="5" t="n"/>
     </row>
     <row r="53">
       <c r="A53" s="5" t="n"/>
@@ -2929,7 +2866,6 @@
       <c r="AG53" s="5" t="n"/>
       <c r="AH53" s="5" t="n"/>
       <c r="AI53" s="5" t="n"/>
-      <c r="AJ53" s="5" t="n"/>
     </row>
     <row r="54">
       <c r="A54" s="5" t="n"/>
@@ -2967,7 +2903,6 @@
       <c r="AG54" s="5" t="n"/>
       <c r="AH54" s="5" t="n"/>
       <c r="AI54" s="5" t="n"/>
-      <c r="AJ54" s="5" t="n"/>
     </row>
     <row r="55">
       <c r="A55" s="5" t="n"/>
@@ -3005,7 +2940,6 @@
       <c r="AG55" s="5" t="n"/>
       <c r="AH55" s="5" t="n"/>
       <c r="AI55" s="5" t="n"/>
-      <c r="AJ55" s="5" t="n"/>
     </row>
     <row r="56">
       <c r="A56" s="5" t="n"/>
@@ -3043,7 +2977,6 @@
       <c r="AG56" s="5" t="n"/>
       <c r="AH56" s="5" t="n"/>
       <c r="AI56" s="5" t="n"/>
-      <c r="AJ56" s="5" t="n"/>
     </row>
     <row r="57">
       <c r="A57" s="5" t="n"/>
@@ -3081,7 +3014,6 @@
       <c r="AG57" s="5" t="n"/>
       <c r="AH57" s="5" t="n"/>
       <c r="AI57" s="5" t="n"/>
-      <c r="AJ57" s="5" t="n"/>
     </row>
     <row r="58">
       <c r="A58" s="5" t="n"/>
@@ -3119,7 +3051,6 @@
       <c r="AG58" s="5" t="n"/>
       <c r="AH58" s="5" t="n"/>
       <c r="AI58" s="5" t="n"/>
-      <c r="AJ58" s="5" t="n"/>
     </row>
     <row r="59">
       <c r="A59" s="5" t="n"/>
@@ -3157,7 +3088,6 @@
       <c r="AG59" s="5" t="n"/>
       <c r="AH59" s="5" t="n"/>
       <c r="AI59" s="5" t="n"/>
-      <c r="AJ59" s="5" t="n"/>
     </row>
     <row r="60">
       <c r="A60" s="5" t="n"/>
@@ -3195,7 +3125,6 @@
       <c r="AG60" s="5" t="n"/>
       <c r="AH60" s="5" t="n"/>
       <c r="AI60" s="5" t="n"/>
-      <c r="AJ60" s="5" t="n"/>
     </row>
     <row r="61">
       <c r="A61" s="5" t="n"/>
@@ -3233,7 +3162,6 @@
       <c r="AG61" s="5" t="n"/>
       <c r="AH61" s="5" t="n"/>
       <c r="AI61" s="5" t="n"/>
-      <c r="AJ61" s="5" t="n"/>
     </row>
     <row r="62">
       <c r="A62" s="5" t="n"/>
@@ -3271,7 +3199,6 @@
       <c r="AG62" s="5" t="n"/>
       <c r="AH62" s="5" t="n"/>
       <c r="AI62" s="5" t="n"/>
-      <c r="AJ62" s="5" t="n"/>
     </row>
     <row r="63">
       <c r="A63" s="5" t="n"/>
@@ -3309,7 +3236,6 @@
       <c r="AG63" s="5" t="n"/>
       <c r="AH63" s="5" t="n"/>
       <c r="AI63" s="5" t="n"/>
-      <c r="AJ63" s="5" t="n"/>
     </row>
     <row r="64">
       <c r="A64" s="5" t="n"/>
@@ -3347,7 +3273,6 @@
       <c r="AG64" s="5" t="n"/>
       <c r="AH64" s="5" t="n"/>
       <c r="AI64" s="5" t="n"/>
-      <c r="AJ64" s="5" t="n"/>
     </row>
     <row r="65">
       <c r="A65" s="5" t="n"/>
@@ -3385,7 +3310,6 @@
       <c r="AG65" s="5" t="n"/>
       <c r="AH65" s="5" t="n"/>
       <c r="AI65" s="5" t="n"/>
-      <c r="AJ65" s="5" t="n"/>
     </row>
     <row r="66">
       <c r="A66" s="5" t="n"/>
@@ -3423,7 +3347,6 @@
       <c r="AG66" s="5" t="n"/>
       <c r="AH66" s="5" t="n"/>
       <c r="AI66" s="5" t="n"/>
-      <c r="AJ66" s="5" t="n"/>
     </row>
     <row r="67">
       <c r="A67" s="5" t="n"/>
@@ -3461,7 +3384,6 @@
       <c r="AG67" s="5" t="n"/>
       <c r="AH67" s="5" t="n"/>
       <c r="AI67" s="5" t="n"/>
-      <c r="AJ67" s="5" t="n"/>
     </row>
     <row r="68">
       <c r="A68" s="5" t="n"/>
@@ -3499,7 +3421,6 @@
       <c r="AG68" s="5" t="n"/>
       <c r="AH68" s="5" t="n"/>
       <c r="AI68" s="5" t="n"/>
-      <c r="AJ68" s="5" t="n"/>
     </row>
     <row r="69">
       <c r="A69" s="5" t="n"/>
@@ -3537,7 +3458,6 @@
       <c r="AG69" s="5" t="n"/>
       <c r="AH69" s="5" t="n"/>
       <c r="AI69" s="5" t="n"/>
-      <c r="AJ69" s="5" t="n"/>
     </row>
     <row r="70">
       <c r="A70" s="5" t="n"/>
@@ -3575,7 +3495,6 @@
       <c r="AG70" s="5" t="n"/>
       <c r="AH70" s="5" t="n"/>
       <c r="AI70" s="5" t="n"/>
-      <c r="AJ70" s="5" t="n"/>
     </row>
     <row r="71">
       <c r="A71" s="5" t="n"/>
@@ -3613,7 +3532,6 @@
       <c r="AG71" s="5" t="n"/>
       <c r="AH71" s="5" t="n"/>
       <c r="AI71" s="5" t="n"/>
-      <c r="AJ71" s="5" t="n"/>
     </row>
     <row r="72">
       <c r="A72" s="5" t="n"/>
@@ -3651,7 +3569,6 @@
       <c r="AG72" s="5" t="n"/>
       <c r="AH72" s="5" t="n"/>
       <c r="AI72" s="5" t="n"/>
-      <c r="AJ72" s="5" t="n"/>
     </row>
     <row r="73">
       <c r="A73" s="5" t="n"/>
@@ -3689,7 +3606,6 @@
       <c r="AG73" s="5" t="n"/>
       <c r="AH73" s="5" t="n"/>
       <c r="AI73" s="5" t="n"/>
-      <c r="AJ73" s="5" t="n"/>
     </row>
     <row r="74">
       <c r="A74" s="5" t="n"/>
@@ -3727,7 +3643,6 @@
       <c r="AG74" s="5" t="n"/>
       <c r="AH74" s="5" t="n"/>
       <c r="AI74" s="5" t="n"/>
-      <c r="AJ74" s="5" t="n"/>
     </row>
     <row r="75">
       <c r="A75" s="5" t="n"/>
@@ -3765,7 +3680,6 @@
       <c r="AG75" s="5" t="n"/>
       <c r="AH75" s="5" t="n"/>
       <c r="AI75" s="5" t="n"/>
-      <c r="AJ75" s="5" t="n"/>
     </row>
     <row r="76">
       <c r="A76" s="5" t="n"/>
@@ -3803,7 +3717,6 @@
       <c r="AG76" s="5" t="n"/>
       <c r="AH76" s="5" t="n"/>
       <c r="AI76" s="5" t="n"/>
-      <c r="AJ76" s="5" t="n"/>
     </row>
     <row r="77">
       <c r="A77" s="5" t="n"/>
@@ -3841,7 +3754,6 @@
       <c r="AG77" s="5" t="n"/>
       <c r="AH77" s="5" t="n"/>
       <c r="AI77" s="5" t="n"/>
-      <c r="AJ77" s="5" t="n"/>
     </row>
     <row r="78">
       <c r="A78" s="5" t="n"/>
@@ -3879,7 +3791,6 @@
       <c r="AG78" s="5" t="n"/>
       <c r="AH78" s="5" t="n"/>
       <c r="AI78" s="5" t="n"/>
-      <c r="AJ78" s="5" t="n"/>
     </row>
     <row r="79">
       <c r="A79" s="5" t="n"/>
@@ -3917,7 +3828,6 @@
       <c r="AG79" s="5" t="n"/>
       <c r="AH79" s="5" t="n"/>
       <c r="AI79" s="5" t="n"/>
-      <c r="AJ79" s="5" t="n"/>
     </row>
     <row r="80">
       <c r="A80" s="5" t="n"/>
@@ -3955,7 +3865,6 @@
       <c r="AG80" s="5" t="n"/>
       <c r="AH80" s="5" t="n"/>
       <c r="AI80" s="5" t="n"/>
-      <c r="AJ80" s="5" t="n"/>
     </row>
     <row r="81">
       <c r="A81" s="5" t="n"/>
@@ -3993,7 +3902,6 @@
       <c r="AG81" s="5" t="n"/>
       <c r="AH81" s="5" t="n"/>
       <c r="AI81" s="5" t="n"/>
-      <c r="AJ81" s="5" t="n"/>
     </row>
     <row r="82">
       <c r="A82" s="5" t="n"/>
@@ -4031,7 +3939,6 @@
       <c r="AG82" s="5" t="n"/>
       <c r="AH82" s="5" t="n"/>
       <c r="AI82" s="5" t="n"/>
-      <c r="AJ82" s="5" t="n"/>
     </row>
     <row r="83">
       <c r="A83" s="5" t="n"/>
@@ -4069,7 +3976,6 @@
       <c r="AG83" s="5" t="n"/>
       <c r="AH83" s="5" t="n"/>
       <c r="AI83" s="5" t="n"/>
-      <c r="AJ83" s="5" t="n"/>
     </row>
     <row r="84">
       <c r="A84" s="5" t="n"/>
@@ -4107,7 +4013,6 @@
       <c r="AG84" s="5" t="n"/>
       <c r="AH84" s="5" t="n"/>
       <c r="AI84" s="5" t="n"/>
-      <c r="AJ84" s="5" t="n"/>
     </row>
     <row r="85">
       <c r="A85" s="5" t="n"/>
@@ -4145,7 +4050,6 @@
       <c r="AG85" s="5" t="n"/>
       <c r="AH85" s="5" t="n"/>
       <c r="AI85" s="5" t="n"/>
-      <c r="AJ85" s="5" t="n"/>
     </row>
     <row r="86">
       <c r="A86" s="5" t="n"/>
@@ -4183,7 +4087,6 @@
       <c r="AG86" s="5" t="n"/>
       <c r="AH86" s="5" t="n"/>
       <c r="AI86" s="5" t="n"/>
-      <c r="AJ86" s="5" t="n"/>
     </row>
     <row r="87">
       <c r="A87" s="5" t="n"/>
@@ -4221,7 +4124,6 @@
       <c r="AG87" s="5" t="n"/>
       <c r="AH87" s="5" t="n"/>
       <c r="AI87" s="5" t="n"/>
-      <c r="AJ87" s="5" t="n"/>
     </row>
     <row r="88">
       <c r="A88" s="5" t="n"/>
@@ -4259,7 +4161,6 @@
       <c r="AG88" s="5" t="n"/>
       <c r="AH88" s="5" t="n"/>
       <c r="AI88" s="5" t="n"/>
-      <c r="AJ88" s="5" t="n"/>
     </row>
     <row r="89">
       <c r="A89" s="5" t="n"/>
@@ -4297,7 +4198,6 @@
       <c r="AG89" s="5" t="n"/>
       <c r="AH89" s="5" t="n"/>
       <c r="AI89" s="5" t="n"/>
-      <c r="AJ89" s="5" t="n"/>
     </row>
     <row r="90">
       <c r="A90" s="5" t="n"/>
@@ -4335,7 +4235,6 @@
       <c r="AG90" s="5" t="n"/>
       <c r="AH90" s="5" t="n"/>
       <c r="AI90" s="5" t="n"/>
-      <c r="AJ90" s="5" t="n"/>
     </row>
     <row r="91">
       <c r="A91" s="5" t="n"/>
@@ -4373,7 +4272,6 @@
       <c r="AG91" s="5" t="n"/>
       <c r="AH91" s="5" t="n"/>
       <c r="AI91" s="5" t="n"/>
-      <c r="AJ91" s="5" t="n"/>
     </row>
     <row r="92">
       <c r="A92" s="5" t="n"/>
@@ -4411,7 +4309,6 @@
       <c r="AG92" s="5" t="n"/>
       <c r="AH92" s="5" t="n"/>
       <c r="AI92" s="5" t="n"/>
-      <c r="AJ92" s="5" t="n"/>
     </row>
     <row r="93">
       <c r="A93" s="5" t="n"/>
@@ -4449,7 +4346,6 @@
       <c r="AG93" s="5" t="n"/>
       <c r="AH93" s="5" t="n"/>
       <c r="AI93" s="5" t="n"/>
-      <c r="AJ93" s="5" t="n"/>
     </row>
     <row r="94">
       <c r="A94" s="5" t="n"/>
@@ -4487,7 +4383,6 @@
       <c r="AG94" s="5" t="n"/>
       <c r="AH94" s="5" t="n"/>
       <c r="AI94" s="5" t="n"/>
-      <c r="AJ94" s="5" t="n"/>
     </row>
     <row r="95">
       <c r="A95" s="5" t="n"/>
@@ -4525,7 +4420,6 @@
       <c r="AG95" s="5" t="n"/>
       <c r="AH95" s="5" t="n"/>
       <c r="AI95" s="5" t="n"/>
-      <c r="AJ95" s="5" t="n"/>
     </row>
     <row r="96">
       <c r="A96" s="5" t="n"/>
@@ -4563,7 +4457,6 @@
       <c r="AG96" s="5" t="n"/>
       <c r="AH96" s="5" t="n"/>
       <c r="AI96" s="5" t="n"/>
-      <c r="AJ96" s="5" t="n"/>
     </row>
     <row r="97">
       <c r="A97" s="5" t="n"/>
@@ -4601,7 +4494,6 @@
       <c r="AG97" s="5" t="n"/>
       <c r="AH97" s="5" t="n"/>
       <c r="AI97" s="5" t="n"/>
-      <c r="AJ97" s="5" t="n"/>
     </row>
     <row r="98">
       <c r="A98" s="5" t="n"/>
@@ -4639,7 +4531,6 @@
       <c r="AG98" s="5" t="n"/>
       <c r="AH98" s="5" t="n"/>
       <c r="AI98" s="5" t="n"/>
-      <c r="AJ98" s="5" t="n"/>
     </row>
     <row r="99">
       <c r="A99" s="5" t="n"/>
@@ -4677,7 +4568,6 @@
       <c r="AG99" s="5" t="n"/>
       <c r="AH99" s="5" t="n"/>
       <c r="AI99" s="5" t="n"/>
-      <c r="AJ99" s="5" t="n"/>
     </row>
     <row r="100">
       <c r="A100" s="5" t="n"/>
@@ -4715,7 +4605,6 @@
       <c r="AG100" s="5" t="n"/>
       <c r="AH100" s="5" t="n"/>
       <c r="AI100" s="5" t="n"/>
-      <c r="AJ100" s="5" t="n"/>
     </row>
     <row r="101">
       <c r="A101" s="5" t="n"/>
@@ -4753,7 +4642,6 @@
       <c r="AG101" s="5" t="n"/>
       <c r="AH101" s="5" t="n"/>
       <c r="AI101" s="5" t="n"/>
-      <c r="AJ101" s="5" t="n"/>
     </row>
     <row r="102">
       <c r="A102" s="5" t="n"/>
@@ -4791,7 +4679,6 @@
       <c r="AG102" s="5" t="n"/>
       <c r="AH102" s="5" t="n"/>
       <c r="AI102" s="5" t="n"/>
-      <c r="AJ102" s="5" t="n"/>
     </row>
     <row r="103">
       <c r="A103" s="5" t="n"/>
@@ -4829,7 +4716,6 @@
       <c r="AG103" s="5" t="n"/>
       <c r="AH103" s="5" t="n"/>
       <c r="AI103" s="5" t="n"/>
-      <c r="AJ103" s="5" t="n"/>
     </row>
     <row r="104">
       <c r="A104" s="5" t="n"/>
@@ -4867,7 +4753,6 @@
       <c r="AG104" s="5" t="n"/>
       <c r="AH104" s="5" t="n"/>
       <c r="AI104" s="5" t="n"/>
-      <c r="AJ104" s="5" t="n"/>
     </row>
     <row r="105">
       <c r="A105" s="5" t="n"/>
@@ -4905,7 +4790,6 @@
       <c r="AG105" s="5" t="n"/>
       <c r="AH105" s="5" t="n"/>
       <c r="AI105" s="5" t="n"/>
-      <c r="AJ105" s="5" t="n"/>
     </row>
     <row r="106">
       <c r="A106" s="5" t="n"/>
@@ -4943,7 +4827,6 @@
       <c r="AG106" s="5" t="n"/>
       <c r="AH106" s="5" t="n"/>
       <c r="AI106" s="5" t="n"/>
-      <c r="AJ106" s="5" t="n"/>
     </row>
     <row r="107">
       <c r="A107" s="5" t="n"/>
@@ -4981,7 +4864,6 @@
       <c r="AG107" s="5" t="n"/>
       <c r="AH107" s="5" t="n"/>
       <c r="AI107" s="5" t="n"/>
-      <c r="AJ107" s="5" t="n"/>
     </row>
     <row r="108">
       <c r="A108" s="5" t="n"/>
@@ -5019,7 +4901,6 @@
       <c r="AG108" s="5" t="n"/>
       <c r="AH108" s="5" t="n"/>
       <c r="AI108" s="5" t="n"/>
-      <c r="AJ108" s="5" t="n"/>
     </row>
     <row r="109">
       <c r="A109" s="5" t="n"/>
@@ -5057,7 +4938,6 @@
       <c r="AG109" s="5" t="n"/>
       <c r="AH109" s="5" t="n"/>
       <c r="AI109" s="5" t="n"/>
-      <c r="AJ109" s="5" t="n"/>
     </row>
     <row r="110">
       <c r="A110" s="5" t="n"/>
@@ -5095,7 +4975,6 @@
       <c r="AG110" s="5" t="n"/>
       <c r="AH110" s="5" t="n"/>
       <c r="AI110" s="5" t="n"/>
-      <c r="AJ110" s="5" t="n"/>
     </row>
     <row r="111">
       <c r="A111" s="5" t="n"/>
@@ -5133,7 +5012,6 @@
       <c r="AG111" s="5" t="n"/>
       <c r="AH111" s="5" t="n"/>
       <c r="AI111" s="5" t="n"/>
-      <c r="AJ111" s="5" t="n"/>
     </row>
     <row r="112">
       <c r="A112" s="5" t="n"/>
@@ -5171,7 +5049,6 @@
       <c r="AG112" s="5" t="n"/>
       <c r="AH112" s="5" t="n"/>
       <c r="AI112" s="5" t="n"/>
-      <c r="AJ112" s="5" t="n"/>
     </row>
     <row r="113">
       <c r="A113" s="5" t="n"/>
@@ -5209,7 +5086,6 @@
       <c r="AG113" s="5" t="n"/>
       <c r="AH113" s="5" t="n"/>
       <c r="AI113" s="5" t="n"/>
-      <c r="AJ113" s="5" t="n"/>
     </row>
     <row r="114">
       <c r="A114" s="5" t="n"/>
@@ -5247,7 +5123,6 @@
       <c r="AG114" s="5" t="n"/>
       <c r="AH114" s="5" t="n"/>
       <c r="AI114" s="5" t="n"/>
-      <c r="AJ114" s="5" t="n"/>
     </row>
     <row r="115">
       <c r="A115" s="5" t="n"/>
@@ -5285,7 +5160,6 @@
       <c r="AG115" s="5" t="n"/>
       <c r="AH115" s="5" t="n"/>
       <c r="AI115" s="5" t="n"/>
-      <c r="AJ115" s="5" t="n"/>
     </row>
     <row r="116">
       <c r="A116" s="5" t="n"/>
@@ -5323,7 +5197,6 @@
       <c r="AG116" s="5" t="n"/>
       <c r="AH116" s="5" t="n"/>
       <c r="AI116" s="5" t="n"/>
-      <c r="AJ116" s="5" t="n"/>
     </row>
     <row r="117">
       <c r="A117" s="5" t="n"/>
@@ -5361,7 +5234,6 @@
       <c r="AG117" s="5" t="n"/>
       <c r="AH117" s="5" t="n"/>
       <c r="AI117" s="5" t="n"/>
-      <c r="AJ117" s="5" t="n"/>
     </row>
     <row r="118">
       <c r="A118" s="5" t="n"/>
@@ -5399,7 +5271,6 @@
       <c r="AG118" s="5" t="n"/>
       <c r="AH118" s="5" t="n"/>
       <c r="AI118" s="5" t="n"/>
-      <c r="AJ118" s="5" t="n"/>
     </row>
     <row r="119">
       <c r="A119" s="5" t="n"/>
@@ -5437,7 +5308,6 @@
       <c r="AG119" s="5" t="n"/>
       <c r="AH119" s="5" t="n"/>
       <c r="AI119" s="5" t="n"/>
-      <c r="AJ119" s="5" t="n"/>
     </row>
     <row r="120">
       <c r="A120" s="5" t="n"/>
@@ -5475,7 +5345,6 @@
       <c r="AG120" s="5" t="n"/>
       <c r="AH120" s="5" t="n"/>
       <c r="AI120" s="5" t="n"/>
-      <c r="AJ120" s="5" t="n"/>
     </row>
     <row r="121">
       <c r="A121" s="5" t="n"/>
@@ -5513,7 +5382,6 @@
       <c r="AG121" s="5" t="n"/>
       <c r="AH121" s="5" t="n"/>
       <c r="AI121" s="5" t="n"/>
-      <c r="AJ121" s="5" t="n"/>
     </row>
     <row r="122">
       <c r="A122" s="5" t="n"/>
@@ -5551,7 +5419,6 @@
       <c r="AG122" s="5" t="n"/>
       <c r="AH122" s="5" t="n"/>
       <c r="AI122" s="5" t="n"/>
-      <c r="AJ122" s="5" t="n"/>
     </row>
     <row r="123">
       <c r="A123" s="5" t="n"/>
@@ -5589,7 +5456,6 @@
       <c r="AG123" s="5" t="n"/>
       <c r="AH123" s="5" t="n"/>
       <c r="AI123" s="5" t="n"/>
-      <c r="AJ123" s="5" t="n"/>
     </row>
     <row r="124">
       <c r="A124" s="5" t="n"/>
@@ -5627,7 +5493,6 @@
       <c r="AG124" s="5" t="n"/>
       <c r="AH124" s="5" t="n"/>
       <c r="AI124" s="5" t="n"/>
-      <c r="AJ124" s="5" t="n"/>
     </row>
     <row r="125">
       <c r="A125" s="5" t="n"/>
@@ -5665,7 +5530,6 @@
       <c r="AG125" s="5" t="n"/>
       <c r="AH125" s="5" t="n"/>
       <c r="AI125" s="5" t="n"/>
-      <c r="AJ125" s="5" t="n"/>
     </row>
     <row r="126">
       <c r="A126" s="5" t="n"/>
@@ -5703,7 +5567,6 @@
       <c r="AG126" s="5" t="n"/>
       <c r="AH126" s="5" t="n"/>
       <c r="AI126" s="5" t="n"/>
-      <c r="AJ126" s="5" t="n"/>
     </row>
     <row r="127">
       <c r="A127" s="5" t="n"/>
@@ -5741,7 +5604,6 @@
       <c r="AG127" s="5" t="n"/>
       <c r="AH127" s="5" t="n"/>
       <c r="AI127" s="5" t="n"/>
-      <c r="AJ127" s="5" t="n"/>
     </row>
     <row r="128">
       <c r="A128" s="5" t="n"/>
@@ -5779,7 +5641,6 @@
       <c r="AG128" s="5" t="n"/>
       <c r="AH128" s="5" t="n"/>
       <c r="AI128" s="5" t="n"/>
-      <c r="AJ128" s="5" t="n"/>
     </row>
     <row r="129">
       <c r="A129" s="5" t="n"/>
@@ -5817,7 +5678,6 @@
       <c r="AG129" s="5" t="n"/>
       <c r="AH129" s="5" t="n"/>
       <c r="AI129" s="5" t="n"/>
-      <c r="AJ129" s="5" t="n"/>
     </row>
     <row r="130">
       <c r="A130" s="5" t="n"/>
@@ -5855,7 +5715,6 @@
       <c r="AG130" s="5" t="n"/>
       <c r="AH130" s="5" t="n"/>
       <c r="AI130" s="5" t="n"/>
-      <c r="AJ130" s="5" t="n"/>
     </row>
     <row r="131">
       <c r="A131" s="5" t="n"/>
@@ -5893,7 +5752,6 @@
       <c r="AG131" s="5" t="n"/>
       <c r="AH131" s="5" t="n"/>
       <c r="AI131" s="5" t="n"/>
-      <c r="AJ131" s="5" t="n"/>
     </row>
     <row r="132">
       <c r="A132" s="5" t="n"/>
@@ -5931,7 +5789,6 @@
       <c r="AG132" s="5" t="n"/>
       <c r="AH132" s="5" t="n"/>
       <c r="AI132" s="5" t="n"/>
-      <c r="AJ132" s="5" t="n"/>
     </row>
     <row r="133">
       <c r="A133" s="5" t="n"/>
@@ -5969,7 +5826,6 @@
       <c r="AG133" s="5" t="n"/>
       <c r="AH133" s="5" t="n"/>
       <c r="AI133" s="5" t="n"/>
-      <c r="AJ133" s="5" t="n"/>
     </row>
     <row r="134">
       <c r="A134" s="5" t="n"/>
@@ -6007,7 +5863,6 @@
       <c r="AG134" s="5" t="n"/>
       <c r="AH134" s="5" t="n"/>
       <c r="AI134" s="5" t="n"/>
-      <c r="AJ134" s="5" t="n"/>
     </row>
     <row r="135">
       <c r="A135" s="5" t="n"/>
@@ -6045,7 +5900,6 @@
       <c r="AG135" s="5" t="n"/>
       <c r="AH135" s="5" t="n"/>
       <c r="AI135" s="5" t="n"/>
-      <c r="AJ135" s="5" t="n"/>
     </row>
     <row r="136">
       <c r="A136" s="5" t="n"/>
@@ -6083,7 +5937,6 @@
       <c r="AG136" s="5" t="n"/>
       <c r="AH136" s="5" t="n"/>
       <c r="AI136" s="5" t="n"/>
-      <c r="AJ136" s="5" t="n"/>
     </row>
     <row r="137">
       <c r="A137" s="5" t="n"/>
@@ -6121,7 +5974,6 @@
       <c r="AG137" s="5" t="n"/>
       <c r="AH137" s="5" t="n"/>
       <c r="AI137" s="5" t="n"/>
-      <c r="AJ137" s="5" t="n"/>
     </row>
     <row r="138">
       <c r="A138" s="5" t="n"/>
@@ -6159,7 +6011,6 @@
       <c r="AG138" s="5" t="n"/>
       <c r="AH138" s="5" t="n"/>
       <c r="AI138" s="5" t="n"/>
-      <c r="AJ138" s="5" t="n"/>
     </row>
     <row r="139">
       <c r="A139" s="5" t="n"/>
@@ -6197,7 +6048,6 @@
       <c r="AG139" s="5" t="n"/>
       <c r="AH139" s="5" t="n"/>
       <c r="AI139" s="5" t="n"/>
-      <c r="AJ139" s="5" t="n"/>
     </row>
     <row r="140">
       <c r="A140" s="5" t="n"/>
@@ -6235,7 +6085,6 @@
       <c r="AG140" s="5" t="n"/>
       <c r="AH140" s="5" t="n"/>
       <c r="AI140" s="5" t="n"/>
-      <c r="AJ140" s="5" t="n"/>
     </row>
     <row r="141">
       <c r="A141" s="5" t="n"/>
@@ -6273,7 +6122,6 @@
       <c r="AG141" s="5" t="n"/>
       <c r="AH141" s="5" t="n"/>
       <c r="AI141" s="5" t="n"/>
-      <c r="AJ141" s="5" t="n"/>
     </row>
     <row r="142">
       <c r="A142" s="5" t="n"/>
@@ -6311,7 +6159,6 @@
       <c r="AG142" s="5" t="n"/>
       <c r="AH142" s="5" t="n"/>
       <c r="AI142" s="5" t="n"/>
-      <c r="AJ142" s="5" t="n"/>
     </row>
     <row r="143">
       <c r="A143" s="5" t="n"/>
@@ -6349,7 +6196,6 @@
       <c r="AG143" s="5" t="n"/>
       <c r="AH143" s="5" t="n"/>
       <c r="AI143" s="5" t="n"/>
-      <c r="AJ143" s="5" t="n"/>
     </row>
     <row r="144">
       <c r="A144" s="5" t="n"/>
@@ -6387,7 +6233,6 @@
       <c r="AG144" s="5" t="n"/>
       <c r="AH144" s="5" t="n"/>
       <c r="AI144" s="5" t="n"/>
-      <c r="AJ144" s="5" t="n"/>
     </row>
     <row r="145">
       <c r="A145" s="5" t="n"/>
@@ -6425,7 +6270,6 @@
       <c r="AG145" s="5" t="n"/>
       <c r="AH145" s="5" t="n"/>
       <c r="AI145" s="5" t="n"/>
-      <c r="AJ145" s="5" t="n"/>
     </row>
     <row r="146">
       <c r="A146" s="5" t="n"/>
@@ -6463,7 +6307,6 @@
       <c r="AG146" s="5" t="n"/>
       <c r="AH146" s="5" t="n"/>
       <c r="AI146" s="5" t="n"/>
-      <c r="AJ146" s="5" t="n"/>
     </row>
     <row r="147">
       <c r="A147" s="5" t="n"/>
@@ -6501,7 +6344,6 @@
       <c r="AG147" s="5" t="n"/>
       <c r="AH147" s="5" t="n"/>
       <c r="AI147" s="5" t="n"/>
-      <c r="AJ147" s="5" t="n"/>
     </row>
     <row r="148">
       <c r="A148" s="5" t="n"/>
@@ -6539,7 +6381,6 @@
       <c r="AG148" s="5" t="n"/>
       <c r="AH148" s="5" t="n"/>
       <c r="AI148" s="5" t="n"/>
-      <c r="AJ148" s="5" t="n"/>
     </row>
     <row r="149">
       <c r="A149" s="5" t="n"/>
@@ -6577,7 +6418,6 @@
       <c r="AG149" s="5" t="n"/>
       <c r="AH149" s="5" t="n"/>
       <c r="AI149" s="5" t="n"/>
-      <c r="AJ149" s="5" t="n"/>
     </row>
     <row r="150">
       <c r="A150" s="5" t="n"/>
@@ -6615,7 +6455,6 @@
       <c r="AG150" s="5" t="n"/>
       <c r="AH150" s="5" t="n"/>
       <c r="AI150" s="5" t="n"/>
-      <c r="AJ150" s="5" t="n"/>
     </row>
     <row r="151">
       <c r="A151" s="5" t="n"/>
@@ -6653,7 +6492,6 @@
       <c r="AG151" s="5" t="n"/>
       <c r="AH151" s="5" t="n"/>
       <c r="AI151" s="5" t="n"/>
-      <c r="AJ151" s="5" t="n"/>
     </row>
     <row r="152">
       <c r="A152" s="5" t="n"/>
@@ -6691,7 +6529,6 @@
       <c r="AG152" s="5" t="n"/>
       <c r="AH152" s="5" t="n"/>
       <c r="AI152" s="5" t="n"/>
-      <c r="AJ152" s="5" t="n"/>
     </row>
     <row r="153">
       <c r="A153" s="5" t="n"/>
@@ -6729,7 +6566,6 @@
       <c r="AG153" s="5" t="n"/>
       <c r="AH153" s="5" t="n"/>
       <c r="AI153" s="5" t="n"/>
-      <c r="AJ153" s="5" t="n"/>
     </row>
     <row r="154">
       <c r="A154" s="5" t="n"/>
@@ -6767,7 +6603,6 @@
       <c r="AG154" s="5" t="n"/>
       <c r="AH154" s="5" t="n"/>
       <c r="AI154" s="5" t="n"/>
-      <c r="AJ154" s="5" t="n"/>
     </row>
     <row r="155">
       <c r="A155" s="5" t="n"/>
@@ -6805,7 +6640,6 @@
       <c r="AG155" s="5" t="n"/>
       <c r="AH155" s="5" t="n"/>
       <c r="AI155" s="5" t="n"/>
-      <c r="AJ155" s="5" t="n"/>
     </row>
     <row r="156">
       <c r="A156" s="5" t="n"/>
@@ -6843,7 +6677,6 @@
       <c r="AG156" s="5" t="n"/>
       <c r="AH156" s="5" t="n"/>
       <c r="AI156" s="5" t="n"/>
-      <c r="AJ156" s="5" t="n"/>
     </row>
     <row r="157">
       <c r="A157" s="5" t="n"/>
@@ -6881,7 +6714,6 @@
       <c r="AG157" s="5" t="n"/>
       <c r="AH157" s="5" t="n"/>
       <c r="AI157" s="5" t="n"/>
-      <c r="AJ157" s="5" t="n"/>
     </row>
     <row r="158">
       <c r="A158" s="5" t="n"/>
@@ -6919,7 +6751,6 @@
       <c r="AG158" s="5" t="n"/>
       <c r="AH158" s="5" t="n"/>
       <c r="AI158" s="5" t="n"/>
-      <c r="AJ158" s="5" t="n"/>
     </row>
     <row r="159">
       <c r="A159" s="5" t="n"/>
@@ -6957,7 +6788,6 @@
       <c r="AG159" s="5" t="n"/>
       <c r="AH159" s="5" t="n"/>
       <c r="AI159" s="5" t="n"/>
-      <c r="AJ159" s="5" t="n"/>
     </row>
     <row r="160">
       <c r="A160" s="5" t="n"/>
@@ -6995,7 +6825,6 @@
       <c r="AG160" s="5" t="n"/>
       <c r="AH160" s="5" t="n"/>
       <c r="AI160" s="5" t="n"/>
-      <c r="AJ160" s="5" t="n"/>
     </row>
     <row r="161">
       <c r="A161" s="5" t="n"/>
@@ -7033,7 +6862,6 @@
       <c r="AG161" s="5" t="n"/>
       <c r="AH161" s="5" t="n"/>
       <c r="AI161" s="5" t="n"/>
-      <c r="AJ161" s="5" t="n"/>
     </row>
     <row r="162">
       <c r="A162" s="5" t="n"/>
@@ -7071,7 +6899,6 @@
       <c r="AG162" s="5" t="n"/>
       <c r="AH162" s="5" t="n"/>
       <c r="AI162" s="5" t="n"/>
-      <c r="AJ162" s="5" t="n"/>
     </row>
     <row r="163">
       <c r="A163" s="5" t="n"/>
@@ -7109,7 +6936,6 @@
       <c r="AG163" s="5" t="n"/>
       <c r="AH163" s="5" t="n"/>
       <c r="AI163" s="5" t="n"/>
-      <c r="AJ163" s="5" t="n"/>
     </row>
     <row r="164">
       <c r="A164" s="5" t="n"/>
@@ -7147,7 +6973,6 @@
       <c r="AG164" s="5" t="n"/>
       <c r="AH164" s="5" t="n"/>
       <c r="AI164" s="5" t="n"/>
-      <c r="AJ164" s="5" t="n"/>
     </row>
     <row r="165">
       <c r="A165" s="5" t="n"/>
@@ -7185,7 +7010,6 @@
       <c r="AG165" s="5" t="n"/>
       <c r="AH165" s="5" t="n"/>
       <c r="AI165" s="5" t="n"/>
-      <c r="AJ165" s="5" t="n"/>
     </row>
     <row r="166">
       <c r="A166" s="5" t="n"/>
@@ -7223,7 +7047,6 @@
       <c r="AG166" s="5" t="n"/>
       <c r="AH166" s="5" t="n"/>
       <c r="AI166" s="5" t="n"/>
-      <c r="AJ166" s="5" t="n"/>
     </row>
     <row r="167">
       <c r="A167" s="5" t="n"/>
@@ -7261,7 +7084,6 @@
       <c r="AG167" s="5" t="n"/>
       <c r="AH167" s="5" t="n"/>
       <c r="AI167" s="5" t="n"/>
-      <c r="AJ167" s="5" t="n"/>
     </row>
     <row r="168">
       <c r="A168" s="5" t="n"/>
@@ -7299,7 +7121,6 @@
       <c r="AG168" s="5" t="n"/>
       <c r="AH168" s="5" t="n"/>
       <c r="AI168" s="5" t="n"/>
-      <c r="AJ168" s="5" t="n"/>
     </row>
     <row r="169">
       <c r="A169" s="5" t="n"/>
@@ -7337,7 +7158,6 @@
       <c r="AG169" s="5" t="n"/>
       <c r="AH169" s="5" t="n"/>
       <c r="AI169" s="5" t="n"/>
-      <c r="AJ169" s="5" t="n"/>
     </row>
     <row r="170">
       <c r="A170" s="5" t="n"/>
@@ -7375,7 +7195,6 @@
       <c r="AG170" s="5" t="n"/>
       <c r="AH170" s="5" t="n"/>
       <c r="AI170" s="5" t="n"/>
-      <c r="AJ170" s="5" t="n"/>
     </row>
     <row r="171">
       <c r="A171" s="5" t="n"/>
@@ -7413,7 +7232,6 @@
       <c r="AG171" s="5" t="n"/>
       <c r="AH171" s="5" t="n"/>
       <c r="AI171" s="5" t="n"/>
-      <c r="AJ171" s="5" t="n"/>
     </row>
     <row r="172">
       <c r="A172" s="5" t="n"/>
@@ -7451,7 +7269,6 @@
       <c r="AG172" s="5" t="n"/>
       <c r="AH172" s="5" t="n"/>
       <c r="AI172" s="5" t="n"/>
-      <c r="AJ172" s="5" t="n"/>
     </row>
     <row r="173">
       <c r="A173" s="5" t="n"/>
@@ -7489,7 +7306,6 @@
       <c r="AG173" s="5" t="n"/>
       <c r="AH173" s="5" t="n"/>
       <c r="AI173" s="5" t="n"/>
-      <c r="AJ173" s="5" t="n"/>
     </row>
     <row r="174">
       <c r="A174" s="5" t="n"/>
@@ -7527,7 +7343,6 @@
       <c r="AG174" s="5" t="n"/>
       <c r="AH174" s="5" t="n"/>
       <c r="AI174" s="5" t="n"/>
-      <c r="AJ174" s="5" t="n"/>
     </row>
     <row r="175">
       <c r="A175" s="5" t="n"/>
@@ -7565,7 +7380,6 @@
       <c r="AG175" s="5" t="n"/>
       <c r="AH175" s="5" t="n"/>
       <c r="AI175" s="5" t="n"/>
-      <c r="AJ175" s="5" t="n"/>
     </row>
     <row r="176">
       <c r="A176" s="5" t="n"/>
@@ -7603,7 +7417,6 @@
       <c r="AG176" s="5" t="n"/>
       <c r="AH176" s="5" t="n"/>
       <c r="AI176" s="5" t="n"/>
-      <c r="AJ176" s="5" t="n"/>
     </row>
     <row r="177">
       <c r="A177" s="5" t="n"/>
@@ -7641,7 +7454,6 @@
       <c r="AG177" s="5" t="n"/>
       <c r="AH177" s="5" t="n"/>
       <c r="AI177" s="5" t="n"/>
-      <c r="AJ177" s="5" t="n"/>
     </row>
     <row r="178">
       <c r="A178" s="5" t="n"/>
@@ -7679,7 +7491,6 @@
       <c r="AG178" s="5" t="n"/>
       <c r="AH178" s="5" t="n"/>
       <c r="AI178" s="5" t="n"/>
-      <c r="AJ178" s="5" t="n"/>
     </row>
     <row r="179">
       <c r="A179" s="5" t="n"/>
@@ -7717,7 +7528,6 @@
       <c r="AG179" s="5" t="n"/>
       <c r="AH179" s="5" t="n"/>
       <c r="AI179" s="5" t="n"/>
-      <c r="AJ179" s="5" t="n"/>
     </row>
     <row r="180">
       <c r="A180" s="5" t="n"/>
@@ -7755,7 +7565,6 @@
       <c r="AG180" s="5" t="n"/>
       <c r="AH180" s="5" t="n"/>
       <c r="AI180" s="5" t="n"/>
-      <c r="AJ180" s="5" t="n"/>
     </row>
     <row r="181">
       <c r="A181" s="5" t="n"/>
@@ -7793,7 +7602,6 @@
       <c r="AG181" s="5" t="n"/>
       <c r="AH181" s="5" t="n"/>
       <c r="AI181" s="5" t="n"/>
-      <c r="AJ181" s="5" t="n"/>
     </row>
     <row r="182">
       <c r="A182" s="5" t="n"/>
@@ -7831,7 +7639,6 @@
       <c r="AG182" s="5" t="n"/>
       <c r="AH182" s="5" t="n"/>
       <c r="AI182" s="5" t="n"/>
-      <c r="AJ182" s="5" t="n"/>
     </row>
     <row r="183">
       <c r="A183" s="5" t="n"/>
@@ -7869,7 +7676,6 @@
       <c r="AG183" s="5" t="n"/>
       <c r="AH183" s="5" t="n"/>
       <c r="AI183" s="5" t="n"/>
-      <c r="AJ183" s="5" t="n"/>
     </row>
     <row r="184">
       <c r="A184" s="5" t="n"/>
@@ -7907,7 +7713,6 @@
       <c r="AG184" s="5" t="n"/>
       <c r="AH184" s="5" t="n"/>
       <c r="AI184" s="5" t="n"/>
-      <c r="AJ184" s="5" t="n"/>
     </row>
     <row r="185">
       <c r="A185" s="5" t="n"/>
@@ -7945,7 +7750,6 @@
       <c r="AG185" s="5" t="n"/>
       <c r="AH185" s="5" t="n"/>
       <c r="AI185" s="5" t="n"/>
-      <c r="AJ185" s="5" t="n"/>
     </row>
     <row r="186">
       <c r="A186" s="5" t="n"/>
@@ -7983,7 +7787,6 @@
       <c r="AG186" s="5" t="n"/>
       <c r="AH186" s="5" t="n"/>
       <c r="AI186" s="5" t="n"/>
-      <c r="AJ186" s="5" t="n"/>
     </row>
     <row r="187">
       <c r="A187" s="5" t="n"/>
@@ -8021,7 +7824,6 @@
       <c r="AG187" s="5" t="n"/>
       <c r="AH187" s="5" t="n"/>
       <c r="AI187" s="5" t="n"/>
-      <c r="AJ187" s="5" t="n"/>
     </row>
     <row r="188">
       <c r="A188" s="5" t="n"/>
@@ -8059,7 +7861,6 @@
       <c r="AG188" s="5" t="n"/>
       <c r="AH188" s="5" t="n"/>
       <c r="AI188" s="5" t="n"/>
-      <c r="AJ188" s="5" t="n"/>
     </row>
     <row r="189">
       <c r="A189" s="5" t="n"/>
@@ -8097,7 +7898,6 @@
       <c r="AG189" s="5" t="n"/>
       <c r="AH189" s="5" t="n"/>
       <c r="AI189" s="5" t="n"/>
-      <c r="AJ189" s="5" t="n"/>
     </row>
     <row r="190">
       <c r="A190" s="5" t="n"/>
@@ -8135,7 +7935,6 @@
       <c r="AG190" s="5" t="n"/>
       <c r="AH190" s="5" t="n"/>
       <c r="AI190" s="5" t="n"/>
-      <c r="AJ190" s="5" t="n"/>
     </row>
     <row r="191">
       <c r="A191" s="5" t="n"/>
@@ -8173,7 +7972,6 @@
       <c r="AG191" s="5" t="n"/>
       <c r="AH191" s="5" t="n"/>
       <c r="AI191" s="5" t="n"/>
-      <c r="AJ191" s="5" t="n"/>
     </row>
     <row r="192">
       <c r="A192" s="5" t="n"/>
@@ -8211,7 +8009,6 @@
       <c r="AG192" s="5" t="n"/>
       <c r="AH192" s="5" t="n"/>
       <c r="AI192" s="5" t="n"/>
-      <c r="AJ192" s="5" t="n"/>
     </row>
     <row r="193">
       <c r="A193" s="5" t="n"/>
@@ -8249,7 +8046,6 @@
       <c r="AG193" s="5" t="n"/>
       <c r="AH193" s="5" t="n"/>
       <c r="AI193" s="5" t="n"/>
-      <c r="AJ193" s="5" t="n"/>
     </row>
     <row r="194">
       <c r="A194" s="5" t="n"/>
@@ -8287,7 +8083,6 @@
       <c r="AG194" s="5" t="n"/>
       <c r="AH194" s="5" t="n"/>
       <c r="AI194" s="5" t="n"/>
-      <c r="AJ194" s="5" t="n"/>
     </row>
     <row r="195">
       <c r="A195" s="5" t="n"/>
@@ -8325,7 +8120,6 @@
       <c r="AG195" s="5" t="n"/>
       <c r="AH195" s="5" t="n"/>
       <c r="AI195" s="5" t="n"/>
-      <c r="AJ195" s="5" t="n"/>
     </row>
     <row r="196">
       <c r="A196" s="5" t="n"/>
@@ -8363,7 +8157,6 @@
       <c r="AG196" s="5" t="n"/>
       <c r="AH196" s="5" t="n"/>
       <c r="AI196" s="5" t="n"/>
-      <c r="AJ196" s="5" t="n"/>
     </row>
     <row r="197">
       <c r="A197" s="5" t="n"/>
@@ -8401,7 +8194,6 @@
       <c r="AG197" s="5" t="n"/>
       <c r="AH197" s="5" t="n"/>
       <c r="AI197" s="5" t="n"/>
-      <c r="AJ197" s="5" t="n"/>
     </row>
     <row r="198">
       <c r="A198" s="5" t="n"/>
@@ -8439,7 +8231,6 @@
       <c r="AG198" s="5" t="n"/>
       <c r="AH198" s="5" t="n"/>
       <c r="AI198" s="5" t="n"/>
-      <c r="AJ198" s="5" t="n"/>
     </row>
     <row r="199">
       <c r="A199" s="5" t="n"/>
@@ -8477,7 +8268,6 @@
       <c r="AG199" s="5" t="n"/>
       <c r="AH199" s="5" t="n"/>
       <c r="AI199" s="5" t="n"/>
-      <c r="AJ199" s="5" t="n"/>
     </row>
     <row r="200">
       <c r="A200" s="5" t="n"/>
@@ -8515,7 +8305,6 @@
       <c r="AG200" s="5" t="n"/>
       <c r="AH200" s="5" t="n"/>
       <c r="AI200" s="5" t="n"/>
-      <c r="AJ200" s="5" t="n"/>
     </row>
     <row r="201">
       <c r="A201" s="5" t="n"/>
@@ -8553,7 +8342,6 @@
       <c r="AG201" s="5" t="n"/>
       <c r="AH201" s="5" t="n"/>
       <c r="AI201" s="5" t="n"/>
-      <c r="AJ201" s="5" t="n"/>
     </row>
     <row r="202">
       <c r="A202" s="5" t="n"/>
@@ -8591,7 +8379,6 @@
       <c r="AG202" s="5" t="n"/>
       <c r="AH202" s="5" t="n"/>
       <c r="AI202" s="5" t="n"/>
-      <c r="AJ202" s="5" t="n"/>
     </row>
     <row r="203">
       <c r="A203" s="5" t="n"/>
@@ -8629,7 +8416,6 @@
       <c r="AG203" s="5" t="n"/>
       <c r="AH203" s="5" t="n"/>
       <c r="AI203" s="5" t="n"/>
-      <c r="AJ203" s="5" t="n"/>
     </row>
   </sheetData>
   <dataValidations count="12">
@@ -8648,6 +8434,9 @@
     <dataValidation sqref="T4:T203" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" error="Numbers only · 请填写数字" type="decimal" operator="greaterThanOrEqual">
       <formula1>0</formula1>
     </dataValidation>
+    <dataValidation sqref="Y4:Y203" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" error="Numbers only · 请填写数字" type="decimal" operator="greaterThanOrEqual">
+      <formula1>0</formula1>
+    </dataValidation>
     <dataValidation sqref="Z4:Z203" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" error="Numbers only · 请填写数字" type="decimal" operator="greaterThanOrEqual">
       <formula1>0</formula1>
     </dataValidation>
@@ -8657,13 +8446,10 @@
     <dataValidation sqref="AB4:AB203" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" error="Numbers only · 请填写数字" type="decimal" operator="greaterThanOrEqual">
       <formula1>0</formula1>
     </dataValidation>
-    <dataValidation sqref="AC4:AC203" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" error="Numbers only · 请填写数字" type="decimal" operator="greaterThanOrEqual">
+    <dataValidation sqref="AD4:AD203" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" error="Numbers only · 请填写数字" type="decimal" operator="greaterThanOrEqual">
       <formula1>0</formula1>
     </dataValidation>
-    <dataValidation sqref="AE4:AE203" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" error="Numbers only · 请填写数字" type="decimal" operator="greaterThanOrEqual">
-      <formula1>0</formula1>
-    </dataValidation>
-    <dataValidation sqref="AD4:AD203" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" error="Numbers only · 请填写数字" type="decimal" operator="greaterThanOrEqual">
+    <dataValidation sqref="AC4:AC203" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" error="Numbers only · 请填写数字" type="decimal" operator="greaterThanOrEqual">
       <formula1>0</formula1>
     </dataValidation>
     <dataValidation sqref="I4:I203" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" error="Numbers only · 请填写数字" type="decimal" operator="greaterThanOrEqual">

</xml_diff>